<commit_message>
Compute Stundenzettel hours with live Excel formulas
Dauer and the net worked time are now written as Excel formulas instead of
pre-computed values, so the sheet recalculates in Excel when a Beginn, Ende
or Pause is edited (the monthly Summe already was a SUM formula). Beginn/Ende/
Pause are HHMM integers, so the formula converts HHMM to a day fraction and
adds a day for overnight shifts via (Ende<=Beginn).

Also drop the template's conditional formatting and its differential format
(the auto-weekday format on column B, which the generator overwrites with
text anyway). ExcelJS mangled that format code to the literal string
"[object Object]" on save, which made Excel flag freshly generated files as
possibly damaged; without the format there is nothing left to corrupt.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ngsi7oTk5AwYFLiNnco1qc
</commit_message>
<xml_diff>
--- a/frontend/public/templates/arbeitszeit-vorlage.xlsx
+++ b/frontend/public/templates/arbeitszeit-vorlage.xlsx
@@ -639,11 +639,7 @@
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{84FF2406-31F1-42CD-9A13-04086DCD9D07}"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <numFmt numFmtId="202" formatCode="ddd\,\ dd;;"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1895,11 +1891,6 @@
     <mergeCell ref="H35:I35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="B11:B42">
-    <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>ISNUMBER($H$7)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.31496062992125984" bottom="0.11811023622047245" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>

</xml_diff>